<commit_message>
Refactor order and mart models to establish bidirectional relationships, update order creation and retrieval logic to use mart IDs, and enhance invoice parsing functionality. Update API configurations and improve error handling in services. Add cascade delete to item alias and update database migrations.
</commit_message>
<xml_diff>
--- a/backend/app/db/seed/data/alias.xlsx
+++ b/backend/app/db/seed/data/alias.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\SupplyChain- mobile\backend\app\db\seed\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1196218A-C541-473C-8D77-24DC8F5CAEFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C61C50BA-9560-47C8-8D10-88BB2616BD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Item_alias" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Item_alias!$D$1:$D$193</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="278">
   <si>
     <t>alias_name</t>
   </si>
@@ -733,13 +736,139 @@
   </si>
   <si>
     <t>RIDGE GOURD</t>
+  </si>
+  <si>
+    <t>Fresh Radish</t>
+  </si>
+  <si>
+    <t>Broccoli</t>
+  </si>
+  <si>
+    <t>Bel Patta (Aegle Marmelos Leaves)</t>
+  </si>
+  <si>
+    <t>Dragon Fruit Red Flesh</t>
+  </si>
+  <si>
+    <t>Raw Banana (Plantains)</t>
+  </si>
+  <si>
+    <t>Holy Tulsi</t>
+  </si>
+  <si>
+    <t>Fresh Brown Coconut (Nariyal)</t>
+  </si>
+  <si>
+    <t>Bullet Green Chilli</t>
+  </si>
+  <si>
+    <t>Spine Gourd (Kakrol)</t>
+  </si>
+  <si>
+    <t>Sweet Potato (Shakarkandi)</t>
+  </si>
+  <si>
+    <t>(Bhartaa Baigan)</t>
+  </si>
+  <si>
+    <t>Valencia orange</t>
+  </si>
+  <si>
+    <t>Indian Plum</t>
+  </si>
+  <si>
+    <t>Fresh Cherry Tomato</t>
+  </si>
+  <si>
+    <t>Blueberry Indian</t>
+  </si>
+  <si>
+    <t>Fresh Red Globe Grapes Packet</t>
+  </si>
+  <si>
+    <t>Red Potato</t>
+  </si>
+  <si>
+    <t>Orange Marigold Flower Per String</t>
+  </si>
+  <si>
+    <t>Groundnut</t>
+  </si>
+  <si>
+    <t>French Beans</t>
+  </si>
+  <si>
+    <t>Green Pumpkin</t>
+  </si>
+  <si>
+    <t>Dasheri Mango</t>
+  </si>
+  <si>
+    <t>Sweet Corn - Packet</t>
+  </si>
+  <si>
+    <t>Fresh Yellow Zucchini</t>
+  </si>
+  <si>
+    <t>Corn Cob</t>
+  </si>
+  <si>
+    <t>Betel Leaves</t>
+  </si>
+  <si>
+    <t>Assorted Fruit (Panch Phal) Combo</t>
+  </si>
+  <si>
+    <t>Guava</t>
+  </si>
+  <si>
+    <t>Fresh Baby Corn</t>
+  </si>
+  <si>
+    <t>Chaunsa Mango</t>
+  </si>
+  <si>
+    <t>BEL PATTA</t>
+  </si>
+  <si>
+    <t>BETEL LEAVES</t>
+  </si>
+  <si>
+    <t>BROCCOLI</t>
+  </si>
+  <si>
+    <t>MANGO CHAUNSA</t>
+  </si>
+  <si>
+    <t>DRAGON FRUIT (RED FLESH)</t>
+  </si>
+  <si>
+    <t>RADISH</t>
+  </si>
+  <si>
+    <t>GROUNDNUT</t>
+  </si>
+  <si>
+    <t>YELLOW ZUCCHINI</t>
+  </si>
+  <si>
+    <t>INDIAN PLUM</t>
+  </si>
+  <si>
+    <t>TULSI</t>
+  </si>
+  <si>
+    <t>MARIGOLD FLOWER</t>
+  </si>
+  <si>
+    <t>SPINE GOURD</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -747,13 +876,35 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -768,8 +919,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1050,7 +1203,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C163"/>
+  <dimension ref="A1:C193"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="34.86328125" bestFit="1" customWidth="1"/>
@@ -1058,56 +1211,56 @@
     <col min="3" max="3" width="27.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>168</v>
+        <v>246</v>
       </c>
       <c r="B2">
-        <v>144046</v>
+        <v>133942</v>
       </c>
       <c r="C2" t="s">
-        <v>222</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B3">
-        <v>133275</v>
+        <v>144046</v>
       </c>
       <c r="C3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>169</v>
       </c>
       <c r="B4">
-        <v>1982</v>
+        <v>133275</v>
       </c>
       <c r="C4" t="s">
-        <v>4</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B5">
-        <v>590000001</v>
+        <v>1982</v>
       </c>
       <c r="C5" t="s">
         <v>4</v>
@@ -1115,164 +1268,161 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>157</v>
+        <v>5</v>
       </c>
       <c r="B6">
-        <v>590000003</v>
+        <v>590000001</v>
       </c>
       <c r="C6" t="s">
-        <v>158</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>157</v>
       </c>
       <c r="B7">
-        <v>590001702</v>
+        <v>590000003</v>
       </c>
       <c r="C7" t="s">
-        <v>6</v>
+        <v>158</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8">
-        <v>590000842</v>
+        <v>590001702</v>
       </c>
       <c r="C8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B9">
-        <v>590000002</v>
+        <v>590000842</v>
       </c>
       <c r="C9" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B10">
-        <v>590000005</v>
+        <v>590000002</v>
       </c>
       <c r="C10" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B11">
-        <v>590000009</v>
+        <v>590000005</v>
       </c>
       <c r="C11" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>170</v>
+        <v>13</v>
       </c>
       <c r="B12">
-        <v>133178</v>
+        <v>590000009</v>
       </c>
       <c r="C12" t="s">
-        <v>224</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>170</v>
       </c>
       <c r="B13">
-        <v>590003579</v>
+        <v>133178</v>
       </c>
       <c r="C13" t="s">
-        <v>15</v>
+        <v>224</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>171</v>
+        <v>262</v>
       </c>
       <c r="B14">
-        <v>147066</v>
-      </c>
-      <c r="C14" t="s">
-        <v>15</v>
+        <v>140348</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15">
-        <v>590004229</v>
+        <v>590003579</v>
       </c>
       <c r="C15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>77</v>
+        <v>171</v>
       </c>
       <c r="B16">
-        <v>590008484</v>
+        <v>147066</v>
       </c>
       <c r="C16" t="s">
-        <v>78</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>172</v>
+        <v>16</v>
       </c>
       <c r="B17">
-        <v>135480</v>
+        <v>590004229</v>
       </c>
       <c r="C17" t="s">
-        <v>225</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>173</v>
+        <v>77</v>
       </c>
       <c r="B18">
-        <v>147002</v>
+        <v>590008484</v>
       </c>
       <c r="C18" t="s">
-        <v>20</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="B19">
-        <v>590000615</v>
+        <v>135480</v>
       </c>
       <c r="C19" t="s">
-        <v>18</v>
+        <v>225</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>173</v>
       </c>
       <c r="B20">
-        <v>590000502</v>
+        <v>147002</v>
       </c>
       <c r="C20" t="s">
         <v>20</v>
@@ -1280,593 +1430,593 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B21">
-        <v>590000454</v>
+        <v>590000615</v>
       </c>
       <c r="C21" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B22">
-        <v>590000129</v>
+        <v>590000502</v>
       </c>
       <c r="C22" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>174</v>
+        <v>21</v>
       </c>
       <c r="B23">
-        <v>133252</v>
+        <v>590000454</v>
       </c>
       <c r="C23" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B24">
-        <v>590003307</v>
+        <v>590000129</v>
       </c>
       <c r="C24" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="B25">
-        <v>147239</v>
+        <v>133252</v>
       </c>
       <c r="C25" t="s">
-        <v>226</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>161</v>
+        <v>238</v>
       </c>
       <c r="B26">
-        <v>149160</v>
+        <v>138574</v>
       </c>
       <c r="C26" t="s">
-        <v>158</v>
+        <v>266</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>159</v>
+        <v>24</v>
       </c>
       <c r="B27">
-        <v>151432</v>
+        <v>590003307</v>
       </c>
       <c r="C27" t="s">
-        <v>55</v>
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>56</v>
+        <v>261</v>
       </c>
       <c r="B28">
-        <v>590000086</v>
+        <v>133614</v>
       </c>
       <c r="C28" t="s">
-        <v>57</v>
+        <v>267</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="B29">
-        <v>135449</v>
+        <v>147239</v>
       </c>
       <c r="C29" t="s">
-        <v>27</v>
+        <v>226</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>26</v>
+        <v>161</v>
       </c>
       <c r="B30">
-        <v>590000173</v>
+        <v>149160</v>
       </c>
       <c r="C30" t="s">
-        <v>27</v>
+        <v>158</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>28</v>
+        <v>159</v>
       </c>
       <c r="B31">
-        <v>590000849</v>
+        <v>151432</v>
       </c>
       <c r="C31" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>162</v>
+        <v>56</v>
       </c>
       <c r="B32">
-        <v>166047</v>
+        <v>590000086</v>
       </c>
       <c r="C32" t="s">
-        <v>31</v>
+        <v>57</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>175</v>
       </c>
       <c r="B33">
-        <v>590000174</v>
+        <v>135449</v>
       </c>
       <c r="C33" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B34">
-        <v>590001217</v>
+        <v>590000173</v>
       </c>
       <c r="C34" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B35">
-        <v>590000582</v>
+        <v>590000849</v>
       </c>
       <c r="C35" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>250</v>
       </c>
       <c r="B36">
-        <v>590000161</v>
+        <v>133256</v>
       </c>
       <c r="C36" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>36</v>
+        <v>162</v>
       </c>
       <c r="B37">
-        <v>590000162</v>
+        <v>166047</v>
       </c>
       <c r="C37" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="B38">
-        <v>590000163</v>
+        <v>590000174</v>
       </c>
       <c r="C38" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B39">
-        <v>590000164</v>
+        <v>590001217</v>
       </c>
       <c r="C39" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>176</v>
+        <v>32</v>
       </c>
       <c r="B40">
-        <v>133229</v>
+        <v>590000582</v>
       </c>
       <c r="C40" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="B41">
-        <v>590000245</v>
+        <v>590000161</v>
       </c>
       <c r="C41" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
-        <v>177</v>
+        <v>36</v>
       </c>
       <c r="B42">
-        <v>133248</v>
+        <v>590000162</v>
       </c>
       <c r="C42" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B43">
-        <v>590000142</v>
+        <v>590000163</v>
       </c>
       <c r="C43" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B44">
-        <v>590000143</v>
+        <v>590000164</v>
       </c>
       <c r="C44" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>45</v>
+        <v>237</v>
       </c>
       <c r="B45">
-        <v>590000144</v>
+        <v>137101</v>
       </c>
       <c r="C45" t="s">
-        <v>46</v>
+        <v>268</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
-        <v>47</v>
+        <v>243</v>
       </c>
       <c r="B46">
-        <v>590000145</v>
+        <v>137103</v>
       </c>
       <c r="C46" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>49</v>
+        <v>176</v>
       </c>
       <c r="B47">
-        <v>590000264</v>
+        <v>133229</v>
       </c>
       <c r="C47" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="B48">
-        <v>590000186</v>
+        <v>590000245</v>
       </c>
       <c r="C48" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B49">
-        <v>134077</v>
+        <v>133248</v>
       </c>
       <c r="C49" t="s">
-        <v>227</v>
+        <v>43</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="B50">
-        <v>590000187</v>
+        <v>590000142</v>
       </c>
       <c r="C50" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="B51">
-        <v>590000175</v>
+        <v>590000143</v>
       </c>
       <c r="C51" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="B52">
-        <v>590000097</v>
+        <v>590000144</v>
       </c>
       <c r="C52" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="B53">
-        <v>590002624</v>
+        <v>590000145</v>
       </c>
       <c r="C53" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
-        <v>179</v>
+        <v>49</v>
       </c>
       <c r="B54">
-        <v>133179</v>
+        <v>590000264</v>
       </c>
       <c r="C54" t="s">
-        <v>229</v>
+        <v>50</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="B55">
-        <v>590000554</v>
+        <v>590000186</v>
       </c>
       <c r="C55" t="s">
-        <v>229</v>
+        <v>52</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B56">
-        <v>133209</v>
+        <v>134077</v>
       </c>
       <c r="C56" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
-        <v>62</v>
+        <v>265</v>
       </c>
       <c r="B57">
-        <v>590000259</v>
+        <v>137986</v>
       </c>
       <c r="C57" t="s">
-        <v>63</v>
+        <v>269</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
-        <v>181</v>
+        <v>53</v>
       </c>
       <c r="B58">
-        <v>133226</v>
+        <v>590000187</v>
       </c>
       <c r="C58" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B59">
-        <v>590000157</v>
+        <v>590000175</v>
       </c>
       <c r="C59" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
-        <v>182</v>
+        <v>55</v>
       </c>
       <c r="B60">
-        <v>141962</v>
+        <v>590000097</v>
       </c>
       <c r="C60" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B61">
-        <v>590000131</v>
+        <v>590002624</v>
       </c>
       <c r="C61" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B62">
-        <v>133206</v>
+        <v>133179</v>
       </c>
       <c r="C62" t="s">
-        <v>69</v>
+        <v>229</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
-        <v>68</v>
+        <v>260</v>
       </c>
       <c r="B63">
-        <v>590000132</v>
+        <v>135531</v>
       </c>
       <c r="C63" t="s">
-        <v>69</v>
+        <v>143</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="B64">
-        <v>590000126</v>
+        <v>590000554</v>
       </c>
       <c r="C64" t="s">
-        <v>71</v>
+        <v>229</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
-        <v>163</v>
+        <v>180</v>
       </c>
       <c r="B65">
-        <v>149160</v>
+        <v>133209</v>
       </c>
       <c r="C65" t="s">
-        <v>158</v>
+        <v>228</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B66">
-        <v>590000034</v>
+        <v>590000259</v>
       </c>
       <c r="C66" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
-        <v>74</v>
+        <v>257</v>
       </c>
       <c r="B67">
-        <v>590004002</v>
+        <v>137987</v>
       </c>
       <c r="C67" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B68">
-        <v>139709</v>
+        <v>133226</v>
       </c>
       <c r="C68" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
-        <v>185</v>
+        <v>239</v>
       </c>
       <c r="B69">
-        <v>135453</v>
+        <v>147541</v>
       </c>
       <c r="C69" t="s">
-        <v>44</v>
+        <v>270</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
-        <v>186</v>
+        <v>255</v>
       </c>
       <c r="B70">
-        <v>133184</v>
+        <v>147212</v>
       </c>
       <c r="C70" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
-        <v>187</v>
+        <v>64</v>
       </c>
       <c r="B71">
-        <v>133180</v>
+        <v>590000157</v>
       </c>
       <c r="C71" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
-        <v>75</v>
+        <v>264</v>
       </c>
       <c r="B72">
-        <v>590000067</v>
+        <v>133223</v>
       </c>
       <c r="C72" t="s">
-        <v>76</v>
+        <v>16</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
-        <v>188</v>
+        <v>242</v>
       </c>
       <c r="B73">
-        <v>146042</v>
+        <v>133176</v>
       </c>
       <c r="C73" t="s">
-        <v>90</v>
+        <v>57</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
-        <v>189</v>
+        <v>249</v>
       </c>
       <c r="B74">
-        <v>133939</v>
+        <v>133194</v>
       </c>
       <c r="C74" t="s">
         <v>148</v>
@@ -1874,986 +2024,1317 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
-        <v>190</v>
+        <v>236</v>
       </c>
       <c r="B75">
-        <v>135450</v>
+        <v>133277</v>
       </c>
       <c r="C75" t="s">
-        <v>230</v>
+        <v>271</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
-        <v>191</v>
+        <v>251</v>
       </c>
       <c r="B76">
-        <v>133266</v>
+        <v>133294</v>
       </c>
       <c r="C76" t="s">
-        <v>153</v>
+        <v>73</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
-        <v>79</v>
+        <v>259</v>
       </c>
       <c r="B77">
-        <v>590009674</v>
+        <v>133232</v>
       </c>
       <c r="C77" t="s">
-        <v>78</v>
+        <v>273</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="B78">
-        <v>135454</v>
+        <v>141962</v>
       </c>
       <c r="C78" t="s">
-        <v>231</v>
+        <v>67</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
-        <v>164</v>
+        <v>66</v>
       </c>
       <c r="B79">
-        <v>152742</v>
+        <v>590000131</v>
       </c>
       <c r="C79" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="B80">
-        <v>151742</v>
+        <v>133206</v>
       </c>
       <c r="C80" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="B81">
-        <v>590000188</v>
+        <v>590000132</v>
       </c>
       <c r="C81" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
-        <v>194</v>
+        <v>70</v>
       </c>
       <c r="B82">
-        <v>136834</v>
+        <v>590000126</v>
       </c>
       <c r="C82" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
-        <v>82</v>
+        <v>163</v>
       </c>
       <c r="B83">
-        <v>590000865</v>
+        <v>149160</v>
       </c>
       <c r="C83" t="s">
-        <v>83</v>
+        <v>158</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
-        <v>195</v>
+        <v>72</v>
       </c>
       <c r="B84">
-        <v>140159</v>
+        <v>590000034</v>
       </c>
       <c r="C84" t="s">
-        <v>38</v>
+        <v>73</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="B85">
-        <v>590000261</v>
+        <v>590004002</v>
       </c>
       <c r="C85" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
-        <v>85</v>
+        <v>184</v>
       </c>
       <c r="B86">
-        <v>590000651</v>
+        <v>139709</v>
       </c>
       <c r="C86" t="s">
-        <v>85</v>
+        <v>36</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
-        <v>86</v>
+        <v>185</v>
       </c>
       <c r="B87">
-        <v>590000660</v>
+        <v>135453</v>
       </c>
       <c r="C87" t="s">
-        <v>86</v>
+        <v>44</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
-        <v>87</v>
+        <v>186</v>
       </c>
       <c r="B88">
-        <v>590001551</v>
+        <v>133184</v>
       </c>
       <c r="C88" t="s">
-        <v>88</v>
+        <v>54</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
-        <v>89</v>
+        <v>187</v>
       </c>
       <c r="B89">
-        <v>590001552</v>
+        <v>133180</v>
       </c>
       <c r="C89" t="s">
-        <v>90</v>
+        <v>63</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
-        <v>91</v>
+        <v>256</v>
       </c>
       <c r="B90">
-        <v>590000656</v>
+        <v>139398</v>
       </c>
       <c r="C90" t="s">
-        <v>91</v>
+        <v>133</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
-        <v>92</v>
+        <v>254</v>
       </c>
       <c r="B91">
-        <v>590000724</v>
+        <v>135484</v>
       </c>
       <c r="C91" t="s">
-        <v>92</v>
+        <v>272</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
-        <v>93</v>
+        <v>263</v>
       </c>
       <c r="B92">
-        <v>590000610</v>
+        <v>133684</v>
       </c>
       <c r="C92" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="B93">
-        <v>590000048</v>
+        <v>590000067</v>
       </c>
       <c r="C93" t="s">
-        <v>96</v>
+        <v>76</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
-        <v>97</v>
+        <v>188</v>
       </c>
       <c r="B94">
-        <v>590000604</v>
+        <v>146042</v>
       </c>
       <c r="C94" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
-        <v>99</v>
+        <v>241</v>
       </c>
       <c r="B95">
-        <v>590000577</v>
+        <v>152757</v>
       </c>
       <c r="C95" t="s">
-        <v>100</v>
+        <v>275</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
-        <v>101</v>
+        <v>189</v>
       </c>
       <c r="B96">
-        <v>590000047</v>
+        <v>133939</v>
       </c>
       <c r="C96" t="s">
-        <v>101</v>
+        <v>148</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
-        <v>196</v>
+        <v>248</v>
       </c>
       <c r="B97">
-        <v>141855</v>
+        <v>146664</v>
       </c>
       <c r="C97" t="s">
-        <v>114</v>
+        <v>274</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="B98">
-        <v>133189</v>
+        <v>135450</v>
       </c>
       <c r="C98" t="s">
-        <v>102</v>
+        <v>230</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
-        <v>102</v>
+        <v>191</v>
       </c>
       <c r="B99">
-        <v>590000532</v>
+        <v>133266</v>
       </c>
       <c r="C99" t="s">
-        <v>102</v>
+        <v>153</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="B100">
-        <v>590001673</v>
+        <v>590009674</v>
       </c>
       <c r="C100" t="s">
-        <v>103</v>
+        <v>78</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
-        <v>104</v>
+        <v>192</v>
       </c>
       <c r="B101">
-        <v>590000051</v>
+        <v>135454</v>
       </c>
       <c r="C101" t="s">
-        <v>105</v>
+        <v>231</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A102" t="s">
-        <v>198</v>
+        <v>164</v>
       </c>
       <c r="B102">
-        <v>133262</v>
+        <v>152742</v>
       </c>
       <c r="C102" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A103" t="s">
-        <v>106</v>
+        <v>193</v>
       </c>
       <c r="B103">
-        <v>590000189</v>
+        <v>151742</v>
       </c>
       <c r="C103" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A104" t="s">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="B104">
-        <v>590000087</v>
+        <v>590000188</v>
       </c>
       <c r="C104" t="s">
-        <v>107</v>
+        <v>81</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A105" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="B105">
-        <v>133269</v>
+        <v>136834</v>
       </c>
       <c r="C105" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A106" t="s">
-        <v>112</v>
+        <v>82</v>
       </c>
       <c r="B106">
-        <v>590002355</v>
+        <v>590000865</v>
       </c>
       <c r="C106" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A107" t="s">
-        <v>108</v>
+        <v>195</v>
       </c>
       <c r="B107">
-        <v>590002741</v>
+        <v>140159</v>
       </c>
       <c r="C107" t="s">
-        <v>107</v>
+        <v>38</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A108" t="s">
-        <v>109</v>
+        <v>84</v>
       </c>
       <c r="B108">
-        <v>590001600</v>
+        <v>590000261</v>
       </c>
       <c r="C108" t="s">
-        <v>107</v>
+        <v>84</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A109" t="s">
-        <v>200</v>
+        <v>85</v>
       </c>
       <c r="B109">
-        <v>133250</v>
+        <v>590000651</v>
       </c>
       <c r="C109" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A110" t="s">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="B110">
-        <v>590000025</v>
+        <v>590000660</v>
       </c>
       <c r="C110" t="s">
-        <v>111</v>
+        <v>86</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A111" t="s">
-        <v>113</v>
+        <v>87</v>
       </c>
       <c r="B111">
-        <v>590001809</v>
+        <v>590001551</v>
       </c>
       <c r="C111" t="s">
-        <v>114</v>
+        <v>88</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A112" t="s">
-        <v>201</v>
+        <v>89</v>
       </c>
       <c r="B112">
-        <v>133222</v>
+        <v>590001552</v>
       </c>
       <c r="C112" t="s">
-        <v>115</v>
+        <v>90</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
-        <v>115</v>
+        <v>91</v>
       </c>
       <c r="B113">
-        <v>590000068</v>
+        <v>590000656</v>
       </c>
       <c r="C113" t="s">
-        <v>115</v>
+        <v>91</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
-        <v>165</v>
+        <v>92</v>
       </c>
       <c r="B114">
-        <v>149158</v>
+        <v>590000724</v>
       </c>
       <c r="C114" t="s">
-        <v>119</v>
+        <v>92</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A115" t="s">
-        <v>116</v>
+        <v>93</v>
       </c>
       <c r="B115">
-        <v>590001297</v>
+        <v>590000610</v>
       </c>
       <c r="C115" t="s">
-        <v>117</v>
+        <v>94</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A116" t="s">
-        <v>118</v>
+        <v>95</v>
       </c>
       <c r="B116">
-        <v>590001296</v>
+        <v>590000048</v>
       </c>
       <c r="C116" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
-        <v>120</v>
+        <v>97</v>
       </c>
       <c r="B117">
-        <v>590001250</v>
+        <v>590000604</v>
       </c>
       <c r="C117" t="s">
-        <v>120</v>
+        <v>98</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
-        <v>202</v>
+        <v>99</v>
       </c>
       <c r="B118">
-        <v>151141</v>
+        <v>590000577</v>
       </c>
       <c r="C118" t="s">
-        <v>8</v>
+        <v>100</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
-        <v>203</v>
+        <v>101</v>
       </c>
       <c r="B119">
-        <v>141854</v>
+        <v>590000047</v>
       </c>
       <c r="C119" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
-        <v>121</v>
+        <v>196</v>
       </c>
       <c r="B120">
-        <v>590000029</v>
+        <v>141855</v>
       </c>
       <c r="C120" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
-        <v>123</v>
+        <v>197</v>
       </c>
       <c r="B121">
-        <v>590000509</v>
+        <v>133189</v>
       </c>
       <c r="C121" t="s">
-        <v>123</v>
+        <v>102</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
-        <v>204</v>
+        <v>102</v>
       </c>
       <c r="B122">
-        <v>133213</v>
+        <v>590000532</v>
       </c>
       <c r="C122" t="s">
-        <v>123</v>
+        <v>102</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
-        <v>205</v>
+        <v>103</v>
       </c>
       <c r="B123">
-        <v>154597</v>
+        <v>590001673</v>
       </c>
       <c r="C123" t="s">
-        <v>125</v>
+        <v>103</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
-        <v>124</v>
+        <v>104</v>
       </c>
       <c r="B124">
-        <v>590000082</v>
+        <v>590000051</v>
       </c>
       <c r="C124" t="s">
-        <v>125</v>
+        <v>105</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
-        <v>126</v>
+        <v>198</v>
       </c>
       <c r="B125">
-        <v>590004194</v>
+        <v>133262</v>
       </c>
       <c r="C125" t="s">
-        <v>125</v>
+        <v>105</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
-        <v>206</v>
+        <v>106</v>
       </c>
       <c r="B126">
-        <v>133599</v>
+        <v>590000189</v>
       </c>
       <c r="C126" t="s">
-        <v>232</v>
+        <v>106</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
       <c r="B127">
-        <v>590000090</v>
+        <v>590000087</v>
       </c>
       <c r="C127" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
-        <v>166</v>
+        <v>199</v>
       </c>
       <c r="B128">
-        <v>157880</v>
+        <v>133269</v>
       </c>
       <c r="C128" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A129" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="B129">
-        <v>590003309</v>
+        <v>590002355</v>
       </c>
       <c r="C129" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A130" t="s">
-        <v>129</v>
+        <v>108</v>
       </c>
       <c r="B130">
-        <v>590000094</v>
+        <v>590002741</v>
       </c>
       <c r="C130" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A131" t="s">
-        <v>130</v>
+        <v>109</v>
       </c>
       <c r="B131">
-        <v>590001787</v>
+        <v>590001600</v>
       </c>
       <c r="C131" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A132" t="s">
-        <v>131</v>
+        <v>200</v>
       </c>
       <c r="B132">
-        <v>590001486</v>
+        <v>133250</v>
       </c>
       <c r="C132" t="s">
-        <v>127</v>
+        <v>52</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A133" t="s">
-        <v>132</v>
+        <v>110</v>
       </c>
       <c r="B133">
-        <v>590000190</v>
+        <v>590000025</v>
       </c>
       <c r="C133" t="s">
-        <v>133</v>
+        <v>111</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A134" t="s">
-        <v>207</v>
+        <v>253</v>
       </c>
       <c r="B134">
-        <v>165548</v>
+        <v>136873</v>
       </c>
       <c r="C134" t="s">
-        <v>147</v>
+        <v>276</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A135" t="s">
-        <v>134</v>
+        <v>113</v>
       </c>
       <c r="B135">
-        <v>590000191</v>
+        <v>590001809</v>
       </c>
       <c r="C135" t="s">
-        <v>135</v>
+        <v>114</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A136" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="B136">
-        <v>133686</v>
+        <v>133222</v>
       </c>
       <c r="C136" t="s">
-        <v>233</v>
+        <v>115</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A137" t="s">
-        <v>209</v>
+        <v>115</v>
       </c>
       <c r="B137">
-        <v>133971</v>
+        <v>590000068</v>
       </c>
       <c r="C137" t="s">
-        <v>234</v>
+        <v>115</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A138" t="s">
-        <v>210</v>
+        <v>165</v>
       </c>
       <c r="B138">
-        <v>152556</v>
+        <v>149158</v>
       </c>
       <c r="C138" t="s">
-        <v>46</v>
+        <v>119</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A139" t="s">
-        <v>211</v>
+        <v>116</v>
       </c>
       <c r="B139">
-        <v>148994</v>
+        <v>590001297</v>
       </c>
       <c r="C139" t="s">
-        <v>10</v>
+        <v>117</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A140" t="s">
-        <v>212</v>
+        <v>118</v>
       </c>
       <c r="B140">
-        <v>133264</v>
+        <v>590001296</v>
       </c>
       <c r="C140" t="s">
-        <v>235</v>
+        <v>119</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A141" t="s">
-        <v>213</v>
+        <v>120</v>
       </c>
       <c r="B141">
-        <v>136870</v>
+        <v>590001250</v>
       </c>
       <c r="C141" t="s">
-        <v>31</v>
+        <v>120</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
-        <v>167</v>
+        <v>202</v>
       </c>
       <c r="B142">
-        <v>160067</v>
+        <v>151141</v>
       </c>
       <c r="C142" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A143" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="B143">
-        <v>134082</v>
+        <v>141854</v>
       </c>
       <c r="C143" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A144" t="s">
-        <v>215</v>
+        <v>121</v>
       </c>
       <c r="B144">
-        <v>147464</v>
+        <v>590000029</v>
       </c>
       <c r="C144" t="s">
-        <v>14</v>
+        <v>122</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
-        <v>216</v>
+        <v>123</v>
       </c>
       <c r="B145">
-        <v>135451</v>
+        <v>590000509</v>
       </c>
       <c r="C145" t="s">
-        <v>137</v>
+        <v>123</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
-        <v>136</v>
+        <v>204</v>
       </c>
       <c r="B146">
-        <v>590000697</v>
+        <v>133213</v>
       </c>
       <c r="C146" t="s">
-        <v>137</v>
+        <v>123</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
-        <v>138</v>
+        <v>205</v>
       </c>
       <c r="B147">
-        <v>590000054</v>
+        <v>154597</v>
       </c>
       <c r="C147" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
-        <v>140</v>
+        <v>124</v>
       </c>
       <c r="B148">
-        <v>590000578</v>
+        <v>590000082</v>
       </c>
       <c r="C148" t="s">
-        <v>141</v>
+        <v>125</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
       <c r="B149">
-        <v>590001511</v>
+        <v>590004194</v>
       </c>
       <c r="C149" t="s">
-        <v>143</v>
+        <v>125</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="B150">
-        <v>147543</v>
+        <v>133599</v>
       </c>
       <c r="C150" t="s">
-        <v>103</v>
+        <v>232</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
-        <v>144</v>
+        <v>127</v>
       </c>
       <c r="B151">
-        <v>590000138</v>
+        <v>590000090</v>
       </c>
       <c r="C151" t="s">
-        <v>145</v>
+        <v>127</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
-        <v>146</v>
+        <v>166</v>
       </c>
       <c r="B152">
-        <v>590001259</v>
+        <v>157880</v>
       </c>
       <c r="C152" t="s">
-        <v>146</v>
+        <v>127</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A153" t="s">
-        <v>218</v>
+        <v>128</v>
       </c>
       <c r="B153">
-        <v>133200</v>
+        <v>590003309</v>
       </c>
       <c r="C153" t="s">
-        <v>146</v>
+        <v>127</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A154" t="s">
-        <v>219</v>
+        <v>129</v>
       </c>
       <c r="B154">
-        <v>151432</v>
+        <v>590000094</v>
       </c>
       <c r="C154" t="s">
-        <v>55</v>
+        <v>127</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A155" t="s">
-        <v>147</v>
+        <v>130</v>
       </c>
       <c r="B155">
-        <v>590000263</v>
+        <v>590001787</v>
       </c>
       <c r="C155" t="s">
-        <v>147</v>
+        <v>127</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A156" t="s">
-        <v>148</v>
+        <v>131</v>
       </c>
       <c r="B156">
-        <v>590000092</v>
+        <v>590001486</v>
       </c>
       <c r="C156" t="s">
-        <v>148</v>
+        <v>127</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A157" t="s">
-        <v>149</v>
+        <v>132</v>
       </c>
       <c r="B157">
-        <v>590000758</v>
+        <v>590000190</v>
       </c>
       <c r="C157" t="s">
-        <v>150</v>
+        <v>133</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A158" t="s">
-        <v>151</v>
+        <v>240</v>
       </c>
       <c r="B158">
-        <v>590000052</v>
+        <v>135447</v>
       </c>
       <c r="C158" t="s">
-        <v>152</v>
+        <v>20</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A159" t="s">
-        <v>153</v>
+        <v>207</v>
       </c>
       <c r="B159">
-        <v>590000692</v>
+        <v>165548</v>
       </c>
       <c r="C159" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A160" t="s">
-        <v>154</v>
+        <v>134</v>
       </c>
       <c r="B160">
-        <v>590009768</v>
+        <v>590000191</v>
       </c>
       <c r="C160" t="s">
-        <v>155</v>
+        <v>135</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A161" t="s">
-        <v>156</v>
+        <v>208</v>
       </c>
       <c r="B161">
-        <v>590000262</v>
+        <v>133686</v>
       </c>
       <c r="C161" t="s">
-        <v>156</v>
+        <v>233</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A162" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="B162">
-        <v>139681</v>
+        <v>133971</v>
       </c>
       <c r="C162" t="s">
-        <v>156</v>
+        <v>234</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A163" t="s">
+        <v>210</v>
+      </c>
+      <c r="B163">
+        <v>152556</v>
+      </c>
+      <c r="C163" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A164" t="s">
+        <v>211</v>
+      </c>
+      <c r="B164">
+        <v>148994</v>
+      </c>
+      <c r="C164" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A165" t="s">
+        <v>252</v>
+      </c>
+      <c r="B165">
+        <v>136835</v>
+      </c>
+      <c r="C165" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A166" t="s">
+        <v>212</v>
+      </c>
+      <c r="B166">
+        <v>133264</v>
+      </c>
+      <c r="C166" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A167" t="s">
+        <v>213</v>
+      </c>
+      <c r="B167">
+        <v>136870</v>
+      </c>
+      <c r="C167" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A168" t="s">
+        <v>167</v>
+      </c>
+      <c r="B168">
+        <v>160067</v>
+      </c>
+      <c r="C168" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="169" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A169" t="s">
+        <v>214</v>
+      </c>
+      <c r="B169">
+        <v>134082</v>
+      </c>
+      <c r="C169" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A170" t="s">
+        <v>215</v>
+      </c>
+      <c r="B170">
+        <v>147464</v>
+      </c>
+      <c r="C170" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A171" t="s">
+        <v>244</v>
+      </c>
+      <c r="B171">
+        <v>136827</v>
+      </c>
+      <c r="C171" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A172" t="s">
+        <v>216</v>
+      </c>
+      <c r="B172">
+        <v>135451</v>
+      </c>
+      <c r="C172" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A173" t="s">
+        <v>136</v>
+      </c>
+      <c r="B173">
+        <v>590000697</v>
+      </c>
+      <c r="C173" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A174" t="s">
+        <v>138</v>
+      </c>
+      <c r="B174">
+        <v>590000054</v>
+      </c>
+      <c r="C174" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A175" t="s">
+        <v>140</v>
+      </c>
+      <c r="B175">
+        <v>590000578</v>
+      </c>
+      <c r="C175" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A176" t="s">
+        <v>258</v>
+      </c>
+      <c r="B176">
+        <v>142007</v>
+      </c>
+      <c r="C176" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A177" t="s">
+        <v>142</v>
+      </c>
+      <c r="B177">
+        <v>590001511</v>
+      </c>
+      <c r="C177" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A178" t="s">
+        <v>217</v>
+      </c>
+      <c r="B178">
+        <v>147543</v>
+      </c>
+      <c r="C178" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A179" t="s">
+        <v>144</v>
+      </c>
+      <c r="B179">
+        <v>590000138</v>
+      </c>
+      <c r="C179" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A180" t="s">
+        <v>245</v>
+      </c>
+      <c r="B180">
+        <v>133196</v>
+      </c>
+      <c r="C180" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A181" t="s">
+        <v>146</v>
+      </c>
+      <c r="B181">
+        <v>590001259</v>
+      </c>
+      <c r="C181" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A182" t="s">
+        <v>218</v>
+      </c>
+      <c r="B182">
+        <v>133200</v>
+      </c>
+      <c r="C182" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A183" t="s">
+        <v>219</v>
+      </c>
+      <c r="B183">
+        <v>151432</v>
+      </c>
+      <c r="C183" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A184" t="s">
+        <v>147</v>
+      </c>
+      <c r="B184">
+        <v>590000263</v>
+      </c>
+      <c r="C184" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A185" t="s">
+        <v>148</v>
+      </c>
+      <c r="B185">
+        <v>590000092</v>
+      </c>
+      <c r="C185" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A186" t="s">
+        <v>247</v>
+      </c>
+      <c r="B186">
+        <v>166780</v>
+      </c>
+      <c r="C186" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A187" t="s">
+        <v>149</v>
+      </c>
+      <c r="B187">
+        <v>590000758</v>
+      </c>
+      <c r="C187" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A188" t="s">
+        <v>151</v>
+      </c>
+      <c r="B188">
+        <v>590000052</v>
+      </c>
+      <c r="C188" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A189" t="s">
+        <v>153</v>
+      </c>
+      <c r="B189">
+        <v>590000692</v>
+      </c>
+      <c r="C189" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A190" t="s">
+        <v>154</v>
+      </c>
+      <c r="B190">
+        <v>590009768</v>
+      </c>
+      <c r="C190" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A191" t="s">
+        <v>156</v>
+      </c>
+      <c r="B191">
+        <v>590000262</v>
+      </c>
+      <c r="C191" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A192" t="s">
+        <v>220</v>
+      </c>
+      <c r="B192">
+        <v>139681</v>
+      </c>
+      <c r="C192" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A193" t="s">
         <v>221</v>
       </c>
-      <c r="B163">
+      <c r="B193">
         <v>152557</v>
       </c>
-      <c r="C163" t="s">
+      <c r="C193" t="s">
         <v>48</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C163">
-    <sortCondition ref="A1:A163"/>
+  <autoFilter ref="D1:D193" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C193">
+    <sortCondition ref="A1:A193"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>